<commit_message>
Train hedonic adjustment on broad table
Keep Gerani as the local comparable source while fitting the hedonic model on a broader committed training table.

Refresh Stavros hedonic report, positioning narrative, and workbook with the split-source workflow.

Tests: python -m compileall tourism_pricing_analytics scripts; python -m unittest discover -s tests
</commit_message>
<xml_diff>
--- a/data/modelling/competitive_pricing_workbook.xlsx
+++ b/data/modelling/competitive_pricing_workbook.xlsx
@@ -99,7 +99,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
@@ -116,7 +116,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source table</t>
+          <t>Comparable source table</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="6">
@@ -128,391 +128,403 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Hedonic training table</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="6">
+        <is>
+          <t>data\modelling\hedonic_training_table.parquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Price unit</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="6">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>EUR/night for a 2-guest Booking.com search</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4"/>
-      <c r="B4" s="6"/>
-    </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5"/>
+      <c r="B5" s="6"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Property</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr" s="6">
-        <is>
-          <t>Stavros Villas &amp; Apartments</t>
-        </is>
-      </c>
+      <c r="B6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="6">
         <is>
-          <t>https://www.booking.com/hotel/gr/stavros-villas-amp-apartments.en-gb.html</t>
+          <t>Stavros Villas &amp; Apartments</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="6">
         <is>
-          <t>Apartment</t>
+          <t>https://www.booking.com/hotel/gr/stavros-villas-amp-apartments.en-gb.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="6">
+        <is>
+          <t>Apartment</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Reference price</t>
         </is>
       </c>
-      <c r="B9" s="4">
+      <c r="B10" s="4">
         <v>133.48</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10"/>
-      <c r="B10" s="6"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr" s="2">
+      <c r="A11"/>
+      <c r="B11" s="6"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
         <is>
           <t>Peer Price Position</t>
         </is>
       </c>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Peer rows</t>
-        </is>
-      </c>
-      <c r="B12" s="6">
-        <v>109</v>
-      </c>
+      <c r="B12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Peer properties with prices</t>
+          <t>Peer rows</t>
         </is>
       </c>
       <c r="B13" s="6">
-        <v>19</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Peer p25</t>
-        </is>
-      </c>
-      <c r="B14" s="4">
-        <v>95.25</v>
+          <t>Peer properties with prices</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Peer median</t>
+          <t>Peer p25</t>
         </is>
       </c>
       <c r="B15" s="4">
-        <v>119.0</v>
+        <v>95.25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Peer p75</t>
+          <t>Peer median</t>
         </is>
       </c>
       <c r="B16" s="4">
-        <v>162.25</v>
+        <v>119.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Subject median</t>
+          <t>Peer p75</t>
         </is>
       </c>
       <c r="B17" s="4">
-        <v>133.48000000000002</v>
+        <v>162.25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Subject percentile vs peers</t>
-        </is>
-      </c>
-      <c r="B18" s="5">
-        <v>0.578</v>
+          <t>Subject median</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <v>133.48000000000002</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gap to peer median</t>
-        </is>
-      </c>
-      <c r="B19" s="4">
-        <v>14.48</v>
+          <t>Subject percentile vs peers</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <v>0.578</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gap to peer median pct</t>
-        </is>
-      </c>
-      <c r="B20" s="5">
-        <v>0.1217</v>
+          <t>Gap to peer median</t>
+        </is>
+      </c>
+      <c r="B20" s="4">
+        <v>14.48</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Gap to peer median pct</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <v>0.1217</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Flags</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr" s="6">
+      <c r="B22" t="inlineStr" s="6">
         <is>
           <t>none</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22"/>
-      <c r="B22" s="6"/>
-    </row>
     <row r="23">
-      <c r="A23" t="inlineStr" s="2">
+      <c r="A23"/>
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="2">
         <is>
           <t>Feature-Adjusted Benchmark</t>
         </is>
       </c>
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Adjusted peer rows</t>
-        </is>
-      </c>
-      <c r="B24" s="6">
-        <v>109</v>
-      </c>
+      <c r="B24" s="2"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Adjusted peer p25</t>
-        </is>
-      </c>
-      <c r="B25" s="4">
-        <v>114.14401759364988</v>
+          <t>Adjusted peer rows</t>
+        </is>
+      </c>
+      <c r="B25" s="6">
+        <v>109</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Adjusted peer median</t>
+          <t>Adjusted peer p25</t>
         </is>
       </c>
       <c r="B26" s="4">
-        <v>120.3503418701948</v>
+        <v>99.18554836537695</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Adjusted peer median</t>
+        </is>
+      </c>
+      <c r="B27" s="4">
+        <v>113.62549015423039</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Adjusted peer p75</t>
         </is>
       </c>
-      <c r="B27" s="4">
-        <v>129.55977905777118</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28"/>
-      <c r="B28" s="6"/>
+      <c r="B28" s="4">
+        <v>130.79983170794557</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr" s="2">
+      <c r="A29"/>
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr" s="2">
         <is>
           <t>Hedonic Training</t>
         </is>
       </c>
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Training rows</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <v>1256</v>
-      </c>
+      <c r="B30" s="2"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Training properties</t>
+          <t>Training rows</t>
         </is>
       </c>
       <c r="B31" s="6">
-        <v>67</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Grouped CV folds</t>
+          <t>Training properties</t>
         </is>
       </c>
       <c r="B32" s="6">
-        <v>5</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GBM mean log R2</t>
+          <t>Grouped CV folds</t>
         </is>
       </c>
       <c r="B33" s="6">
-        <v>-1.6276315989865757</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GBM mean log MAE</t>
+          <t>GBM mean log R2</t>
         </is>
       </c>
       <c r="B34" s="6">
-        <v>0.383152815729961</v>
+        <v>0.3108050369803198</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GBM mean EUR/night MAE</t>
-        </is>
-      </c>
-      <c r="B35" s="4">
-        <v>83.3125819910135</v>
+          <t>GBM mean log MAE</t>
+        </is>
+      </c>
+      <c r="B35" s="6">
+        <v>0.2851139151161721</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OLS R2</t>
-        </is>
-      </c>
-      <c r="B36" s="6">
-        <v>0.8668255626390471</v>
+          <t>GBM mean EUR/night MAE</t>
+        </is>
+      </c>
+      <c r="B36" s="4">
+        <v>53.32149472419017</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>OLS R2</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <v>0.6246570229449309</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>OLS condition number</t>
         </is>
       </c>
-      <c r="B37" s="6">
-        <v>1.1247963270357698e+16</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38"/>
-      <c r="B38" s="6"/>
+      <c r="B38" s="6">
+        <v>9.448097188104942e+16</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr" s="2">
+      <c r="A39"/>
+      <c r="B39" s="6"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr" s="2">
         <is>
           <t>Price Gap Decomposition</t>
         </is>
       </c>
-      <c r="B39" s="2"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Client observed price</t>
-        </is>
-      </c>
-      <c r="B40" s="4">
-        <v>117.86</v>
-      </c>
+      <c r="B40" s="2"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Competitor observed price</t>
+          <t>Client observed price</t>
         </is>
       </c>
       <c r="B41" s="4">
-        <v>57.0</v>
+        <v>117.86</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Observed gap</t>
+          <t>Competitor observed price</t>
         </is>
       </c>
       <c r="B42" s="4">
-        <v>60.86</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Feature-explained gap</t>
+          <t>Observed gap</t>
         </is>
       </c>
       <c r="B43" s="4">
-        <v>59.97577158285408</v>
+        <v>60.86</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Feature-explained gap</t>
+        </is>
+      </c>
+      <c r="B44" s="4">
+        <v>35.79981320938094</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Residual gap</t>
         </is>
       </c>
-      <c r="B44" s="4">
-        <v>0.8842284171459198</v>
+      <c r="B45" s="4">
+        <v>25.060186790619056</v>
       </c>
     </row>
   </sheetData>
@@ -7310,16 +7322,16 @@
         <v>108.0</v>
       </c>
       <c r="K4" s="4">
-        <v>113.89000568434557</v>
+        <v>159.76552449754183</v>
       </c>
       <c r="L4" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M4" s="6">
-        <v>1.0777489841273864</v>
+        <v>0.8366202276729348</v>
       </c>
       <c r="N4" s="4">
-        <v>116.39689028575773</v>
+        <v>90.35498458867696</v>
       </c>
     </row>
     <row r="5">
@@ -7368,16 +7380,16 @@
         <v>108.0</v>
       </c>
       <c r="K5" s="4">
-        <v>114.88542199838649</v>
+        <v>159.76552449754183</v>
       </c>
       <c r="L5" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M5" s="6">
-        <v>1.0684109070887131</v>
+        <v>0.8366202276729348</v>
       </c>
       <c r="N5" s="4">
-        <v>115.38837796558101</v>
+        <v>90.35498458867696</v>
       </c>
     </row>
     <row r="6">
@@ -7426,16 +7438,16 @@
         <v>109.25</v>
       </c>
       <c r="K6" s="4">
-        <v>118.01807343709262</v>
+        <v>169.36024625036478</v>
       </c>
       <c r="L6" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M6" s="6">
-        <v>1.0412296785409456</v>
+        <v>0.8080410429188393</v>
       </c>
       <c r="N6" s="4">
-        <v>113.7543423805983</v>
+        <v>88.27848393888318</v>
       </c>
     </row>
     <row r="7">
@@ -7484,16 +7496,16 @@
         <v>98.0</v>
       </c>
       <c r="K7" s="4">
-        <v>104.65585606761886</v>
+        <v>161.09504804553345</v>
       </c>
       <c r="L7" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M7" s="6">
-        <v>1.1728425196699879</v>
+        <v>0.8297155691690751</v>
       </c>
       <c r="N7" s="4">
-        <v>114.93856692765881</v>
+        <v>81.31212577856935</v>
       </c>
     </row>
     <row r="8">
@@ -7542,16 +7554,16 @@
         <v>67.0</v>
       </c>
       <c r="K8" s="4">
-        <v>72.174717089582</v>
+        <v>80.91214979625612</v>
       </c>
       <c r="L8" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M8" s="6">
-        <v>1.7006625433143983</v>
+        <v>1.651953010963058</v>
       </c>
       <c r="N8" s="4">
-        <v>113.94439040206468</v>
+        <v>110.6808517345249</v>
       </c>
     </row>
     <row r="9">
@@ -7600,16 +7612,16 @@
         <v>67.0</v>
       </c>
       <c r="K9" s="4">
-        <v>72.04849027209481</v>
+        <v>80.91214979625612</v>
       </c>
       <c r="L9" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M9" s="6">
-        <v>1.7036420536365653</v>
+        <v>1.651953010963058</v>
       </c>
       <c r="N9" s="4">
-        <v>114.14401759364988</v>
+        <v>110.6808517345249</v>
       </c>
     </row>
     <row r="10">
@@ -7658,16 +7670,16 @@
         <v>397.0</v>
       </c>
       <c r="K10" s="4">
-        <v>323.69235948765885</v>
+        <v>264.0379161331309</v>
       </c>
       <c r="L10" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M10" s="6">
-        <v>0.37963182344318125</v>
+        <v>0.5182968871036494</v>
       </c>
       <c r="N10" s="4">
-        <v>150.71383390694297</v>
+        <v>205.7638641801488</v>
       </c>
     </row>
     <row r="11">
@@ -7716,16 +7728,16 @@
         <v>312.0</v>
       </c>
       <c r="K11" s="4">
-        <v>323.69235948765885</v>
+        <v>264.0379161331309</v>
       </c>
       <c r="L11" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M11" s="6">
-        <v>0.37963182344318125</v>
+        <v>0.5182968871036494</v>
       </c>
       <c r="N11" s="4">
-        <v>118.44512891427254</v>
+        <v>161.70862877633863</v>
       </c>
     </row>
     <row r="12">
@@ -7774,16 +7786,16 @@
         <v>359.0</v>
       </c>
       <c r="K12" s="4">
-        <v>309.1970711478095</v>
+        <v>247.28879874441662</v>
       </c>
       <c r="L12" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M12" s="6">
-        <v>0.3974291225034983</v>
+        <v>0.5534016530630507</v>
       </c>
       <c r="N12" s="4">
-        <v>142.6770549787559</v>
+        <v>198.67119344963518</v>
       </c>
     </row>
     <row r="13">
@@ -7832,16 +7844,16 @@
         <v>265.5</v>
       </c>
       <c r="K13" s="4">
-        <v>309.1970711478095</v>
+        <v>247.28879874441662</v>
       </c>
       <c r="L13" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M13" s="6">
-        <v>0.3974291225034983</v>
+        <v>0.5534016530630507</v>
       </c>
       <c r="N13" s="4">
-        <v>105.51743202467881</v>
+        <v>146.92813888823994</v>
       </c>
     </row>
     <row r="14">
@@ -7890,16 +7902,16 @@
         <v>94.0</v>
       </c>
       <c r="K14" s="4">
-        <v>96.03966857849892</v>
+        <v>112.22666603798459</v>
       </c>
       <c r="L14" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M14" s="6">
-        <v>1.2780639473806499</v>
+        <v>1.191009892730657</v>
       </c>
       <c r="N14" s="4">
-        <v>120.13801105378109</v>
+        <v>111.95492991668175</v>
       </c>
     </row>
     <row r="15">
@@ -7948,16 +7960,16 @@
         <v>84.75</v>
       </c>
       <c r="K15" s="4">
-        <v>94.15556545540535</v>
+        <v>112.22666603798459</v>
       </c>
       <c r="L15" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M15" s="6">
-        <v>1.3036386891723466</v>
+        <v>1.191009892730657</v>
       </c>
       <c r="N15" s="4">
-        <v>110.48337890735637</v>
+        <v>100.93808840892318</v>
       </c>
     </row>
     <row r="16">
@@ -8006,16 +8018,16 @@
         <v>105.5</v>
       </c>
       <c r="K16" s="4">
-        <v>97.4321138962438</v>
+        <v>110.00185161043224</v>
       </c>
       <c r="L16" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M16" s="6">
-        <v>1.259798571744811</v>
+        <v>1.215098359914726</v>
       </c>
       <c r="N16" s="4">
-        <v>132.90874931907757</v>
+        <v>128.19287697100359</v>
       </c>
     </row>
     <row r="17">
@@ -8064,16 +8076,16 @@
         <v>95.25</v>
       </c>
       <c r="K17" s="4">
-        <v>94.99389487743872</v>
+        <v>110.00185161043224</v>
       </c>
       <c r="L17" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M17" s="6">
-        <v>1.292133963839795</v>
+        <v>1.215098359914726</v>
       </c>
       <c r="N17" s="4">
-        <v>123.07576005574047</v>
+        <v>115.73811878187766</v>
       </c>
     </row>
     <row r="18">
@@ -8122,16 +8134,16 @@
         <v>94.0</v>
       </c>
       <c r="K18" s="4">
-        <v>95.26304885932275</v>
+        <v>113.57728926038003</v>
       </c>
       <c r="L18" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M18" s="6">
-        <v>1.2884831988720618</v>
+        <v>1.1768468005341444</v>
       </c>
       <c r="N18" s="4">
-        <v>121.1174206939738</v>
+        <v>110.62359925020957</v>
       </c>
     </row>
     <row r="19">
@@ -8180,16 +8192,16 @@
         <v>84.75</v>
       </c>
       <c r="K19" s="4">
-        <v>92.87911025602502</v>
+        <v>113.57728926038003</v>
       </c>
       <c r="L19" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M19" s="6">
-        <v>1.3215548425282564</v>
+        <v>1.1768468005341444</v>
       </c>
       <c r="N19" s="4">
-        <v>112.00177290426973</v>
+        <v>99.73776634526874</v>
       </c>
     </row>
     <row r="20">
@@ -8238,16 +8250,16 @@
         <v>94.0</v>
       </c>
       <c r="K20" s="4">
-        <v>96.03966857849892</v>
+        <v>112.22666603798459</v>
       </c>
       <c r="L20" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M20" s="6">
-        <v>1.2780639473806499</v>
+        <v>1.191009892730657</v>
       </c>
       <c r="N20" s="4">
-        <v>120.13801105378109</v>
+        <v>111.95492991668175</v>
       </c>
     </row>
     <row r="21">
@@ -8296,16 +8308,16 @@
         <v>84.86</v>
       </c>
       <c r="K21" s="4">
-        <v>94.15556545540535</v>
+        <v>112.22666603798459</v>
       </c>
       <c r="L21" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M21" s="6">
-        <v>1.3036386891723466</v>
+        <v>1.191009892730657</v>
       </c>
       <c r="N21" s="4">
-        <v>110.62677916316534</v>
+        <v>101.06909949712355</v>
       </c>
     </row>
     <row r="22">
@@ -8354,16 +8366,16 @@
         <v>105.57</v>
       </c>
       <c r="K22" s="4">
-        <v>97.4321138962438</v>
+        <v>110.00185161043224</v>
       </c>
       <c r="L22" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M22" s="6">
-        <v>1.259798571744811</v>
+        <v>1.215098359914726</v>
       </c>
       <c r="N22" s="4">
-        <v>132.9969352190997</v>
+        <v>128.27793385619762</v>
       </c>
     </row>
     <row r="23">
@@ -8412,16 +8424,16 @@
         <v>95.14</v>
       </c>
       <c r="K23" s="4">
-        <v>94.99389487743872</v>
+        <v>110.00185161043224</v>
       </c>
       <c r="L23" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M23" s="6">
-        <v>1.292133963839795</v>
+        <v>1.215098359914726</v>
       </c>
       <c r="N23" s="4">
-        <v>122.9336253197181</v>
+        <v>115.60445796228703</v>
       </c>
     </row>
     <row r="24">
@@ -8470,16 +8482,16 @@
         <v>94.0</v>
       </c>
       <c r="K24" s="4">
-        <v>95.26304885932275</v>
+        <v>113.57728926038003</v>
       </c>
       <c r="L24" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M24" s="6">
-        <v>1.2884831988720618</v>
+        <v>1.1768468005341444</v>
       </c>
       <c r="N24" s="4">
-        <v>121.1174206939738</v>
+        <v>110.62359925020957</v>
       </c>
     </row>
     <row r="25">
@@ -8528,16 +8540,16 @@
         <v>84.86</v>
       </c>
       <c r="K25" s="4">
-        <v>92.87911025602502</v>
+        <v>113.57728926038003</v>
       </c>
       <c r="L25" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M25" s="6">
-        <v>1.3215548425282564</v>
+        <v>1.1768468005341444</v>
       </c>
       <c r="N25" s="4">
-        <v>112.14714393694784</v>
+        <v>99.8672194933275</v>
       </c>
     </row>
     <row r="26">
@@ -8586,16 +8598,16 @@
         <v>94.0</v>
       </c>
       <c r="K26" s="4">
-        <v>96.03966857849892</v>
+        <v>115.58397887994236</v>
       </c>
       <c r="L26" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M26" s="6">
-        <v>1.279512127496414</v>
+        <v>1.1839878790752045</v>
       </c>
       <c r="N26" s="4">
-        <v>120.27413998466292</v>
+        <v>111.29486063306922</v>
       </c>
     </row>
     <row r="27">
@@ -8644,16 +8656,16 @@
         <v>84.75</v>
       </c>
       <c r="K27" s="4">
-        <v>94.26225355810983</v>
+        <v>115.58397887994236</v>
       </c>
       <c r="L27" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M27" s="6">
-        <v>1.3036386891723466</v>
+        <v>1.1839878790752045</v>
       </c>
       <c r="N27" s="4">
-        <v>110.48337890735637</v>
+        <v>100.34297275162358</v>
       </c>
     </row>
     <row r="28">
@@ -8702,16 +8714,16 @@
         <v>105.5</v>
       </c>
       <c r="K28" s="4">
-        <v>97.60366316364556</v>
+        <v>114.53332534144914</v>
       </c>
       <c r="L28" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M28" s="6">
-        <v>1.2590093105511253</v>
+        <v>1.1948490066201782</v>
       </c>
       <c r="N28" s="4">
-        <v>132.82548226314373</v>
+        <v>126.0565701984288</v>
       </c>
     </row>
     <row r="29">
@@ -8760,16 +8772,16 @@
         <v>95.25</v>
       </c>
       <c r="K29" s="4">
-        <v>95.26897869546248</v>
+        <v>114.53332534144914</v>
       </c>
       <c r="L29" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M29" s="6">
-        <v>1.289862895032572</v>
+        <v>1.1948490066201782</v>
       </c>
       <c r="N29" s="4">
-        <v>122.85944075185247</v>
+        <v>113.80936788057198</v>
       </c>
     </row>
     <row r="30">
@@ -8818,16 +8830,16 @@
         <v>94.0</v>
       </c>
       <c r="K30" s="4">
-        <v>96.03966857849892</v>
+        <v>115.58397887994236</v>
       </c>
       <c r="L30" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M30" s="6">
-        <v>1.279512127496414</v>
+        <v>1.1839878790752045</v>
       </c>
       <c r="N30" s="4">
-        <v>120.27413998466292</v>
+        <v>111.29486063306922</v>
       </c>
     </row>
     <row r="31">
@@ -8876,16 +8888,16 @@
         <v>84.86</v>
       </c>
       <c r="K31" s="4">
-        <v>94.26225355810983</v>
+        <v>115.58397887994236</v>
       </c>
       <c r="L31" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M31" s="6">
-        <v>1.3036386891723466</v>
+        <v>1.1839878790752045</v>
       </c>
       <c r="N31" s="4">
-        <v>110.62677916316534</v>
+        <v>100.47321141832185</v>
       </c>
     </row>
     <row r="32">
@@ -8934,16 +8946,16 @@
         <v>105.57</v>
       </c>
       <c r="K32" s="4">
-        <v>97.60366316364556</v>
+        <v>114.53332534144914</v>
       </c>
       <c r="L32" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M32" s="6">
-        <v>1.2590093105511253</v>
+        <v>1.1948490066201782</v>
       </c>
       <c r="N32" s="4">
-        <v>132.9136129148823</v>
+        <v>126.14020962889221</v>
       </c>
     </row>
     <row r="33">
@@ -8992,16 +9004,16 @@
         <v>95.14</v>
       </c>
       <c r="K33" s="4">
-        <v>95.26897869546248</v>
+        <v>114.53332534144914</v>
       </c>
       <c r="L33" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M33" s="6">
-        <v>1.289862895032572</v>
+        <v>1.1948490066201782</v>
       </c>
       <c r="N33" s="4">
-        <v>122.71755583339889</v>
+        <v>113.67793448984376</v>
       </c>
     </row>
     <row r="34">
@@ -9050,16 +9062,16 @@
         <v>78.25</v>
       </c>
       <c r="K34" s="4">
-        <v>93.96918490138768</v>
+        <v>137.07818020641773</v>
       </c>
       <c r="L34" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M34" s="6">
-        <v>1.306224354902892</v>
+        <v>0.9750864016296696</v>
       </c>
       <c r="N34" s="4">
-        <v>102.2120557711513</v>
+        <v>76.30051092752164</v>
       </c>
     </row>
     <row r="35">
@@ -9108,16 +9120,16 @@
         <v>162.0</v>
       </c>
       <c r="K35" s="4">
-        <v>140.0016160383906</v>
+        <v>169.49337450969628</v>
       </c>
       <c r="L35" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M35" s="6">
-        <v>0.8777321587004324</v>
+        <v>0.8074063685675652</v>
       </c>
       <c r="N35" s="4">
-        <v>142.19260970947005</v>
+        <v>130.79983170794557</v>
       </c>
     </row>
     <row r="36">
@@ -9166,16 +9178,16 @@
         <v>162.0</v>
       </c>
       <c r="K36" s="4">
-        <v>139.756766329958</v>
+        <v>169.49337450969628</v>
       </c>
       <c r="L36" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M36" s="6">
-        <v>0.8792699194027109</v>
+        <v>0.8074063685675652</v>
       </c>
       <c r="N36" s="4">
-        <v>142.44172694323916</v>
+        <v>130.79983170794557</v>
       </c>
     </row>
     <row r="37">
@@ -9224,16 +9236,16 @@
         <v>57.0</v>
       </c>
       <c r="K37" s="4">
-        <v>62.76906634571162</v>
+        <v>97.86325627003833</v>
       </c>
       <c r="L37" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M37" s="6">
-        <v>1.955498863923306</v>
+        <v>1.365814653771554</v>
       </c>
       <c r="N37" s="4">
-        <v>111.46343524362844</v>
+        <v>77.85143526497858</v>
       </c>
     </row>
     <row r="38">
@@ -9282,16 +9294,16 @@
         <v>57.0</v>
       </c>
       <c r="K38" s="4">
-        <v>62.76906634571162</v>
+        <v>97.86325627003833</v>
       </c>
       <c r="L38" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M38" s="6">
-        <v>1.955498863923306</v>
+        <v>1.365814653771554</v>
       </c>
       <c r="N38" s="4">
-        <v>111.46343524362844</v>
+        <v>77.85143526497858</v>
       </c>
     </row>
     <row r="39">
@@ -9340,16 +9352,16 @@
         <v>104.5</v>
       </c>
       <c r="K39" s="4">
-        <v>116.87592762370659</v>
+        <v>138.65658333877644</v>
       </c>
       <c r="L39" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M39" s="6">
-        <v>1.0514048800755824</v>
+        <v>0.9869710237614442</v>
       </c>
       <c r="N39" s="4">
-        <v>109.87180996789836</v>
+        <v>103.13847198307091</v>
       </c>
     </row>
     <row r="40">
@@ -9398,16 +9410,16 @@
         <v>292.0</v>
       </c>
       <c r="K40" s="4">
-        <v>238.68141028008677</v>
+        <v>193.5507743994551</v>
       </c>
       <c r="L40" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M40" s="6">
-        <v>0.5142622451598876</v>
+        <v>0.6905840077062259</v>
       </c>
       <c r="N40" s="4">
-        <v>150.1645755866872</v>
+        <v>201.65053025021794</v>
       </c>
     </row>
     <row r="41">
@@ -9456,16 +9468,16 @@
         <v>237.0</v>
       </c>
       <c r="K41" s="4">
-        <v>238.68141028008677</v>
+        <v>193.5507743994551</v>
       </c>
       <c r="L41" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M41" s="6">
-        <v>0.5142622451598876</v>
+        <v>0.6905840077062259</v>
       </c>
       <c r="N41" s="4">
-        <v>121.88015210289336</v>
+        <v>163.66840982637552</v>
       </c>
     </row>
     <row r="42">
@@ -9514,16 +9526,16 @@
         <v>148.25</v>
       </c>
       <c r="K42" s="4">
-        <v>142.4737245110662</v>
+        <v>144.5534797662274</v>
       </c>
       <c r="L42" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M42" s="6">
-        <v>0.8625023392111929</v>
+        <v>0.946708652261092</v>
       </c>
       <c r="N42" s="4">
-        <v>127.86597178805935</v>
+        <v>140.3495576977069</v>
       </c>
     </row>
     <row r="43">
@@ -9572,16 +9584,16 @@
         <v>155.5</v>
       </c>
       <c r="K43" s="4">
-        <v>142.4737245110662</v>
+        <v>144.5534797662274</v>
       </c>
       <c r="L43" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M43" s="6">
-        <v>0.8625023392111929</v>
+        <v>0.946708652261092</v>
       </c>
       <c r="N43" s="4">
-        <v>134.1191137473405</v>
+        <v>147.2131954265998</v>
       </c>
     </row>
     <row r="44">
@@ -9630,16 +9642,16 @@
         <v>126.25</v>
       </c>
       <c r="K44" s="4">
-        <v>134.97903810085595</v>
+        <v>135.96498312721945</v>
       </c>
       <c r="L44" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M44" s="6">
-        <v>0.9103926238910307</v>
+        <v>1.0065093736751958</v>
       </c>
       <c r="N44" s="4">
-        <v>114.93706876624263</v>
+        <v>127.07180842649346</v>
       </c>
     </row>
     <row r="45">
@@ -9688,16 +9700,16 @@
         <v>148.14</v>
       </c>
       <c r="K45" s="4">
-        <v>141.90927719537683</v>
+        <v>144.5534797662274</v>
       </c>
       <c r="L45" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M45" s="6">
-        <v>0.865932961505698</v>
+        <v>0.946708652261092</v>
       </c>
       <c r="N45" s="4">
-        <v>128.27930891745407</v>
+        <v>140.24541974595815</v>
       </c>
     </row>
     <row r="46">
@@ -9746,16 +9758,16 @@
         <v>155.57</v>
       </c>
       <c r="K46" s="4">
-        <v>141.90927719537683</v>
+        <v>144.5534797662274</v>
       </c>
       <c r="L46" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M46" s="6">
-        <v>0.865932961505698</v>
+        <v>0.946708652261092</v>
       </c>
       <c r="N46" s="4">
-        <v>134.71319082144143</v>
+        <v>147.2794650322581</v>
       </c>
     </row>
     <row r="47">
@@ -9804,16 +9816,16 @@
         <v>126.29</v>
       </c>
       <c r="K47" s="4">
-        <v>134.97903810085595</v>
+        <v>135.96498312721945</v>
       </c>
       <c r="L47" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M47" s="6">
-        <v>0.9103926238910307</v>
+        <v>1.0065093736751958</v>
       </c>
       <c r="N47" s="4">
-        <v>114.97348447119828</v>
+        <v>127.11206880144049</v>
       </c>
     </row>
     <row r="48">
@@ -9862,16 +9874,16 @@
         <v>96.5</v>
       </c>
       <c r="K48" s="4">
-        <v>105.66355841979203</v>
+        <v>141.03401096560432</v>
       </c>
       <c r="L48" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M48" s="6">
-        <v>1.1629735218524313</v>
+        <v>0.9703335321187984</v>
       </c>
       <c r="N48" s="4">
-        <v>112.22694485875962</v>
+        <v>93.63718584946405</v>
       </c>
     </row>
     <row r="49">
@@ -9920,16 +9932,16 @@
         <v>99.5</v>
       </c>
       <c r="K49" s="4">
-        <v>105.85735190575747</v>
+        <v>141.03401096560432</v>
       </c>
       <c r="L49" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M49" s="6">
-        <v>1.160844461481774</v>
+        <v>0.9703335321187984</v>
       </c>
       <c r="N49" s="4">
-        <v>115.5040239174365</v>
+        <v>96.54818644582043</v>
       </c>
     </row>
     <row r="50">
@@ -9978,16 +9990,16 @@
         <v>100.43</v>
       </c>
       <c r="K50" s="4">
-        <v>105.66355841979203</v>
+        <v>141.03401096560432</v>
       </c>
       <c r="L50" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M50" s="6">
-        <v>1.1629735218524313</v>
+        <v>0.9703335321187984</v>
       </c>
       <c r="N50" s="4">
-        <v>116.79743079963968</v>
+        <v>97.45059663069092</v>
       </c>
     </row>
     <row r="51">
@@ -10036,16 +10048,16 @@
         <v>103.43</v>
       </c>
       <c r="K51" s="4">
-        <v>105.85735190575747</v>
+        <v>141.03401096560432</v>
       </c>
       <c r="L51" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M51" s="6">
-        <v>1.160844461481774</v>
+        <v>0.9703335321187984</v>
       </c>
       <c r="N51" s="4">
-        <v>120.06614265105988</v>
+        <v>100.36159722704733</v>
       </c>
     </row>
     <row r="52">
@@ -10094,16 +10106,16 @@
         <v>127.5</v>
       </c>
       <c r="K52" s="4">
-        <v>140.63790213457088</v>
+        <v>199.10000053971513</v>
       </c>
       <c r="L52" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M52" s="6">
-        <v>0.8727721052829414</v>
+        <v>0.6713363592018528</v>
       </c>
       <c r="N52" s="4">
-        <v>111.27844342357503</v>
+        <v>85.59538579823622</v>
       </c>
     </row>
     <row r="53">
@@ -10152,16 +10164,16 @@
         <v>114.0</v>
       </c>
       <c r="K53" s="4">
-        <v>140.17026592564633</v>
+        <v>197.9361580715072</v>
       </c>
       <c r="L53" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M53" s="6">
-        <v>0.875683848625043</v>
+        <v>0.6752837418978882</v>
       </c>
       <c r="N53" s="4">
-        <v>99.8279587432549</v>
+        <v>76.98234657635925</v>
       </c>
     </row>
     <row r="54">
@@ -10210,16 +10222,16 @@
         <v>141.0</v>
       </c>
       <c r="K54" s="4">
-        <v>140.63790213457088</v>
+        <v>199.10000053971513</v>
       </c>
       <c r="L54" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M54" s="6">
-        <v>0.8727721052829414</v>
+        <v>0.6713363592018528</v>
       </c>
       <c r="N54" s="4">
-        <v>123.06086684489473</v>
+        <v>94.65842664746124</v>
       </c>
     </row>
     <row r="55">
@@ -10268,16 +10280,16 @@
         <v>161.0</v>
       </c>
       <c r="K55" s="4">
-        <v>152.7041136628763</v>
+        <v>221.41082210362913</v>
       </c>
       <c r="L55" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M55" s="6">
-        <v>0.8047191245824298</v>
+        <v>0.6180819379510045</v>
       </c>
       <c r="N55" s="4">
-        <v>129.55977905777118</v>
+        <v>99.51119201011173</v>
       </c>
     </row>
     <row r="56">
@@ -10326,16 +10338,16 @@
         <v>147.5</v>
       </c>
       <c r="K56" s="4">
-        <v>152.19635599786105</v>
+        <v>220.11656134528408</v>
       </c>
       <c r="L56" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M56" s="6">
-        <v>0.8074038294888787</v>
+        <v>0.6217161906071551</v>
       </c>
       <c r="N56" s="4">
-        <v>119.0920648496096</v>
+        <v>91.70313811455537</v>
       </c>
     </row>
     <row r="57">
@@ -10384,16 +10396,16 @@
         <v>174.5</v>
       </c>
       <c r="K57" s="4">
-        <v>152.7041136628763</v>
+        <v>221.41082210362913</v>
       </c>
       <c r="L57" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M57" s="6">
-        <v>0.8047191245824298</v>
+        <v>0.6180819379510045</v>
       </c>
       <c r="N57" s="4">
-        <v>140.423487239634</v>
+        <v>107.85529817245029</v>
       </c>
     </row>
     <row r="58">
@@ -10442,16 +10454,16 @@
         <v>174.25</v>
       </c>
       <c r="K58" s="4">
-        <v>166.57212208415493</v>
+        <v>165.15338178273944</v>
       </c>
       <c r="L58" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M58" s="6">
-        <v>0.7368870396365187</v>
+        <v>0.8093268695839003</v>
       </c>
       <c r="N58" s="4">
-        <v>128.4025666566634</v>
+        <v>141.02520702499464</v>
       </c>
     </row>
     <row r="59">
@@ -10500,16 +10512,16 @@
         <v>193.25</v>
       </c>
       <c r="K59" s="4">
-        <v>166.57212208415493</v>
+        <v>165.15338178273944</v>
       </c>
       <c r="L59" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M59" s="6">
-        <v>0.7368870396365187</v>
+        <v>0.8093268695839003</v>
       </c>
       <c r="N59" s="4">
-        <v>142.40342040975725</v>
+        <v>156.40241754708873</v>
       </c>
     </row>
     <row r="60">
@@ -10558,16 +10570,16 @@
         <v>93.75</v>
       </c>
       <c r="K60" s="4">
-        <v>109.09371084818066</v>
+        <v>146.02245920024416</v>
       </c>
       <c r="L60" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M60" s="6">
-        <v>1.1264070101890293</v>
+        <v>0.9371848053967535</v>
       </c>
       <c r="N60" s="4">
-        <v>105.6006572052215</v>
+        <v>87.86107550594565</v>
       </c>
     </row>
     <row r="61">
@@ -10616,16 +10628,16 @@
         <v>105.0</v>
       </c>
       <c r="K61" s="4">
-        <v>108.66150727900911</v>
+        <v>146.02245920024416</v>
       </c>
       <c r="L61" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M61" s="6">
-        <v>1.1308873191994089</v>
+        <v>0.9371848053967535</v>
       </c>
       <c r="N61" s="4">
-        <v>118.74316851593794</v>
+        <v>98.40440456665912</v>
       </c>
     </row>
     <row r="62">
@@ -10674,16 +10686,16 @@
         <v>98.5</v>
       </c>
       <c r="K62" s="4">
-        <v>108.14636321883161</v>
+        <v>128.95914476387685</v>
       </c>
       <c r="L62" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M62" s="6">
-        <v>1.134988124197893</v>
+        <v>1.036476084919416</v>
       </c>
       <c r="N62" s="4">
-        <v>111.79633023349245</v>
+        <v>102.09289436456247</v>
       </c>
     </row>
     <row r="63">
@@ -10732,16 +10744,16 @@
         <v>103.75</v>
       </c>
       <c r="K63" s="4">
-        <v>114.83344650851977</v>
+        <v>143.14777553222757</v>
       </c>
       <c r="L63" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M63" s="6">
-        <v>1.0701056565241087</v>
+        <v>0.9560052854494163</v>
       </c>
       <c r="N63" s="4">
-        <v>111.02346186437627</v>
+        <v>99.18554836537695</v>
       </c>
     </row>
     <row r="64">
@@ -10790,16 +10802,16 @@
         <v>268.5</v>
       </c>
       <c r="K64" s="4">
-        <v>247.72251424661061</v>
+        <v>177.3028997780227</v>
       </c>
       <c r="L64" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M64" s="6">
-        <v>0.49605471283321995</v>
+        <v>0.7718431575595653</v>
       </c>
       <c r="N64" s="4">
-        <v>133.19069039571954</v>
+        <v>207.2398878047433</v>
       </c>
     </row>
     <row r="65">
@@ -10848,16 +10860,16 @@
         <v>269.5</v>
       </c>
       <c r="K65" s="4">
-        <v>247.72251424661061</v>
+        <v>177.3028997780227</v>
       </c>
       <c r="L65" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M65" s="6">
-        <v>0.49605471283321995</v>
+        <v>0.7718431575595653</v>
       </c>
       <c r="N65" s="4">
-        <v>133.68674510855277</v>
+        <v>208.01173096230286</v>
       </c>
     </row>
     <row r="66">
@@ -10906,16 +10918,16 @@
         <v>213.25</v>
       </c>
       <c r="K66" s="4">
-        <v>232.09214493713023</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L66" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M66" s="6">
-        <v>0.5294617820875102</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N66" s="4">
-        <v>112.90772503016154</v>
+        <v>175.3108160766125</v>
       </c>
     </row>
     <row r="67">
@@ -10964,16 +10976,16 @@
         <v>214.0</v>
       </c>
       <c r="K67" s="4">
-        <v>232.09214493713023</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L67" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M67" s="6">
-        <v>0.5294617820875102</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N67" s="4">
-        <v>113.30482136672717</v>
+        <v>175.92738401123128</v>
       </c>
     </row>
     <row r="68">
@@ -11022,16 +11034,16 @@
         <v>271.14</v>
       </c>
       <c r="K68" s="4">
-        <v>247.28927078055773</v>
+        <v>177.3028997780227</v>
       </c>
       <c r="L68" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M68" s="6">
-        <v>0.4969237859736007</v>
+        <v>0.7718431575595653</v>
       </c>
       <c r="N68" s="4">
-        <v>134.7359153288821</v>
+        <v>209.27755374070054</v>
       </c>
     </row>
     <row r="69">
@@ -11080,16 +11092,16 @@
         <v>272.29</v>
       </c>
       <c r="K69" s="4">
-        <v>247.28927078055773</v>
+        <v>177.3028997780227</v>
       </c>
       <c r="L69" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M69" s="6">
-        <v>0.4969237859736007</v>
+        <v>0.7718431575595653</v>
       </c>
       <c r="N69" s="4">
-        <v>135.30737768275173</v>
+        <v>210.16517337189407</v>
       </c>
     </row>
     <row r="70">
@@ -11138,16 +11150,16 @@
         <v>253.57</v>
       </c>
       <c r="K70" s="4">
-        <v>236.34612724541662</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L70" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M70" s="6">
-        <v>0.5199320255386529</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N70" s="4">
-        <v>131.8391637158362</v>
+        <v>208.45750824171924</v>
       </c>
     </row>
     <row r="71">
@@ -11196,16 +11208,16 @@
         <v>254.57</v>
       </c>
       <c r="K71" s="4">
-        <v>236.34612724541662</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L71" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M71" s="6">
-        <v>0.5199320255386529</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N71" s="4">
-        <v>132.35909574137486</v>
+        <v>209.27959882121098</v>
       </c>
     </row>
     <row r="72">
@@ -11254,16 +11266,16 @@
         <v>215.43</v>
       </c>
       <c r="K72" s="4">
-        <v>232.09214493713023</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L72" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M72" s="6">
-        <v>0.5294617820875102</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N72" s="4">
-        <v>114.06195171511231</v>
+        <v>177.1029735399045</v>
       </c>
     </row>
     <row r="73">
@@ -11312,16 +11324,16 @@
         <v>216.29</v>
       </c>
       <c r="K73" s="4">
-        <v>232.09214493713023</v>
+        <v>166.4658778765534</v>
       </c>
       <c r="L73" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M73" s="6">
-        <v>0.5294617820875102</v>
+        <v>0.822090579491735</v>
       </c>
       <c r="N73" s="4">
-        <v>114.51728884770756</v>
+        <v>177.80997143826735</v>
       </c>
     </row>
     <row r="74">
@@ -11370,16 +11382,16 @@
         <v>145.25</v>
       </c>
       <c r="K74" s="4">
-        <v>153.74316538311908</v>
+        <v>170.06009663053555</v>
       </c>
       <c r="L74" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M74" s="6">
-        <v>0.7983758993298509</v>
+        <v>0.7859755000010924</v>
       </c>
       <c r="N74" s="4">
-        <v>115.96409937766084</v>
+        <v>114.16294137515867</v>
       </c>
     </row>
     <row r="75">
@@ -11428,16 +11440,16 @@
         <v>184.75</v>
       </c>
       <c r="K75" s="4">
-        <v>166.4951347878498</v>
+        <v>185.3932137216464</v>
       </c>
       <c r="L75" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M75" s="6">
-        <v>0.7372277759645574</v>
+        <v>0.720970669833169</v>
       </c>
       <c r="N75" s="4">
-        <v>136.20283160945198</v>
+        <v>133.199331251678</v>
       </c>
     </row>
     <row r="76">
@@ -11486,16 +11498,16 @@
         <v>161.0</v>
       </c>
       <c r="K76" s="4">
-        <v>153.74316538311908</v>
+        <v>170.06009663053555</v>
       </c>
       <c r="L76" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M76" s="6">
-        <v>0.7983758993298509</v>
+        <v>0.7859755000010924</v>
       </c>
       <c r="N76" s="4">
-        <v>128.538519792106</v>
+        <v>126.54205550017588</v>
       </c>
     </row>
     <row r="77">
@@ -11544,16 +11556,16 @@
         <v>145.14</v>
       </c>
       <c r="K77" s="4">
-        <v>153.74316538311908</v>
+        <v>170.06009663053555</v>
       </c>
       <c r="L77" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M77" s="6">
-        <v>0.7983758993298509</v>
+        <v>0.7859755000010924</v>
       </c>
       <c r="N77" s="4">
-        <v>115.87627802873455</v>
+        <v>114.07648407015854</v>
       </c>
     </row>
     <row r="78">
@@ -11602,16 +11614,16 @@
         <v>184.71</v>
       </c>
       <c r="K78" s="4">
-        <v>165.83552030645086</v>
+        <v>185.3932137216464</v>
       </c>
       <c r="L78" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M78" s="6">
-        <v>0.7401601158891834</v>
+        <v>0.720970669833169</v>
       </c>
       <c r="N78" s="4">
-        <v>136.71497500589106</v>
+        <v>133.17049242488466</v>
       </c>
     </row>
     <row r="79">
@@ -11660,16 +11672,16 @@
         <v>161.0</v>
       </c>
       <c r="K79" s="4">
-        <v>153.74316538311908</v>
+        <v>170.06009663053555</v>
       </c>
       <c r="L79" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M79" s="6">
-        <v>0.7983758993298509</v>
+        <v>0.7859755000010924</v>
       </c>
       <c r="N79" s="4">
-        <v>128.538519792106</v>
+        <v>126.54205550017588</v>
       </c>
     </row>
     <row r="80">
@@ -11718,16 +11730,16 @@
         <v>169.0</v>
       </c>
       <c r="K80" s="4">
-        <v>175.76549845944535</v>
+        <v>186.31710450169973</v>
       </c>
       <c r="L80" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M80" s="6">
-        <v>0.6991356195839473</v>
+        <v>0.7345006266340283</v>
       </c>
       <c r="N80" s="4">
-        <v>118.1539197096871</v>
+        <v>124.13060590115077</v>
       </c>
     </row>
     <row r="81">
@@ -11776,16 +11788,16 @@
         <v>215.25</v>
       </c>
       <c r="K81" s="4">
-        <v>189.4046710658608</v>
+        <v>203.11600110357506</v>
       </c>
       <c r="L81" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M81" s="6">
-        <v>0.6487903385666546</v>
+        <v>0.673753073443742</v>
       </c>
       <c r="N81" s="4">
-        <v>139.6521203764724</v>
+        <v>145.02534905876547</v>
       </c>
     </row>
     <row r="82">
@@ -11834,16 +11846,16 @@
         <v>187.5</v>
       </c>
       <c r="K82" s="4">
-        <v>189.4046710658608</v>
+        <v>203.11600110357506</v>
       </c>
       <c r="L82" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M82" s="6">
-        <v>0.6487903385666546</v>
+        <v>0.673753073443742</v>
       </c>
       <c r="N82" s="4">
-        <v>121.64818848124773</v>
+        <v>126.32870127070163</v>
       </c>
     </row>
     <row r="83">
@@ -11892,16 +11904,16 @@
         <v>127.5</v>
       </c>
       <c r="K83" s="4">
-        <v>152.97719997110767</v>
+        <v>207.3118842825195</v>
       </c>
       <c r="L83" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M83" s="6">
-        <v>0.8032825851835069</v>
+        <v>0.6601166666482099</v>
       </c>
       <c r="N83" s="4">
-        <v>102.41852961089714</v>
+        <v>84.16487499764676</v>
       </c>
     </row>
     <row r="84">
@@ -11950,16 +11962,16 @@
         <v>162.25</v>
       </c>
       <c r="K84" s="4">
-        <v>165.66563765737328</v>
+        <v>225.19267012523204</v>
       </c>
       <c r="L84" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M84" s="6">
-        <v>0.7417586555944209</v>
+        <v>0.6077019733059359</v>
       </c>
       <c r="N84" s="4">
-        <v>120.3503418701948</v>
+        <v>98.5996451688881</v>
       </c>
     </row>
     <row r="85">
@@ -12008,16 +12020,16 @@
         <v>141.25</v>
       </c>
       <c r="K85" s="4">
-        <v>165.66563765737328</v>
+        <v>225.19267012523204</v>
       </c>
       <c r="L85" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M85" s="6">
-        <v>0.7417586555944209</v>
+        <v>0.6077019733059359</v>
       </c>
       <c r="N85" s="4">
-        <v>104.77341010271195</v>
+        <v>85.83790372946345</v>
       </c>
     </row>
     <row r="86">
@@ -12066,16 +12078,16 @@
         <v>169.14</v>
       </c>
       <c r="K86" s="4">
-        <v>175.76549845944535</v>
+        <v>186.31710450169973</v>
       </c>
       <c r="L86" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M86" s="6">
-        <v>0.6991356195839473</v>
+        <v>0.7345006266340283</v>
       </c>
       <c r="N86" s="4">
-        <v>118.25179869642884</v>
+        <v>124.23343598887953</v>
       </c>
     </row>
     <row r="87">
@@ -12124,16 +12136,16 @@
         <v>215.29</v>
       </c>
       <c r="K87" s="4">
-        <v>188.65429440146858</v>
+        <v>203.11600110357506</v>
       </c>
       <c r="L87" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M87" s="6">
-        <v>0.6513709166112102</v>
+        <v>0.673753073443742</v>
       </c>
       <c r="N87" s="4">
-        <v>140.23364463722743</v>
+        <v>145.0522991817032</v>
       </c>
     </row>
     <row r="88">
@@ -12182,16 +12194,16 @@
         <v>187.57</v>
       </c>
       <c r="K88" s="4">
-        <v>188.65429440146858</v>
+        <v>203.11600110357506</v>
       </c>
       <c r="L88" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M88" s="6">
-        <v>0.6513709166112102</v>
+        <v>0.673753073443742</v>
       </c>
       <c r="N88" s="4">
-        <v>122.17764282876469</v>
+        <v>126.37586398584268</v>
       </c>
     </row>
     <row r="89">
@@ -12240,16 +12252,16 @@
         <v>83.0</v>
       </c>
       <c r="K89" s="4">
-        <v>91.60017368131598</v>
+        <v>140.1205598713433</v>
       </c>
       <c r="L89" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M89" s="6">
-        <v>1.3400066069263623</v>
+        <v>0.9539147545666875</v>
       </c>
       <c r="N89" s="4">
-        <v>111.22054837488807</v>
+        <v>79.17492462903506</v>
       </c>
     </row>
     <row r="90">
@@ -12298,16 +12310,16 @@
         <v>83.0</v>
       </c>
       <c r="K90" s="4">
-        <v>91.60017368131598</v>
+        <v>140.1205598713433</v>
       </c>
       <c r="L90" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M90" s="6">
-        <v>1.3400066069263623</v>
+        <v>0.9539147545666875</v>
       </c>
       <c r="N90" s="4">
-        <v>111.22054837488807</v>
+        <v>79.17492462903506</v>
       </c>
     </row>
     <row r="91">
@@ -12356,16 +12368,16 @@
         <v>92.0</v>
       </c>
       <c r="K91" s="4">
-        <v>92.66534141137483</v>
+        <v>144.1490568315369</v>
       </c>
       <c r="L91" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M91" s="6">
-        <v>1.3246035255366637</v>
+        <v>0.9272559419908497</v>
       </c>
       <c r="N91" s="4">
-        <v>121.86352434937307</v>
+        <v>85.30754666315818</v>
       </c>
     </row>
     <row r="92">
@@ -12414,16 +12426,16 @@
         <v>92.0</v>
       </c>
       <c r="K92" s="4">
-        <v>92.66534141137483</v>
+        <v>144.1490568315369</v>
       </c>
       <c r="L92" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M92" s="6">
-        <v>1.3246035255366637</v>
+        <v>0.9272559419908497</v>
       </c>
       <c r="N92" s="4">
-        <v>121.86352434937307</v>
+        <v>85.30754666315818</v>
       </c>
     </row>
     <row r="93">
@@ -12472,16 +12484,16 @@
         <v>92.0</v>
       </c>
       <c r="K93" s="4">
-        <v>97.58237466892555</v>
+        <v>156.52756401825053</v>
       </c>
       <c r="L93" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M93" s="6">
-        <v>1.2592839750399847</v>
+        <v>0.874287099958829</v>
       </c>
       <c r="N93" s="4">
-        <v>115.85412570367859</v>
+        <v>80.43441319621228</v>
       </c>
     </row>
     <row r="94">
@@ -12530,16 +12542,16 @@
         <v>104.5</v>
       </c>
       <c r="K94" s="4">
-        <v>102.0776915134187</v>
+        <v>155.1174166681702</v>
       </c>
       <c r="L94" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M94" s="6">
-        <v>1.203827387209005</v>
+        <v>0.882235102599008</v>
       </c>
       <c r="N94" s="4">
-        <v>125.79996196334103</v>
+        <v>92.19356822159634</v>
       </c>
     </row>
     <row r="95">
@@ -12588,16 +12600,16 @@
         <v>92.0</v>
       </c>
       <c r="K95" s="4">
-        <v>97.19577630049312</v>
+        <v>156.52756401825053</v>
       </c>
       <c r="L95" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M95" s="6">
-        <v>1.2642928051422149</v>
+        <v>0.874287099958829</v>
       </c>
       <c r="N95" s="4">
-        <v>116.31493807308377</v>
+        <v>80.43441319621228</v>
       </c>
     </row>
     <row r="96">
@@ -12646,16 +12658,16 @@
         <v>107.71</v>
       </c>
       <c r="K96" s="4">
-        <v>101.67328375918721</v>
+        <v>155.1174166681702</v>
       </c>
       <c r="L96" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M96" s="6">
-        <v>1.2086156374960384</v>
+        <v>0.882235102599008</v>
       </c>
       <c r="N96" s="4">
-        <v>130.1799903146983</v>
+        <v>95.02554290093914</v>
       </c>
     </row>
     <row r="97">
@@ -12704,16 +12716,16 @@
         <v>112.0</v>
       </c>
       <c r="K97" s="4">
-        <v>106.23382292548273</v>
+        <v>128.66089802326437</v>
       </c>
       <c r="L97" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M97" s="6">
-        <v>1.1554214519293404</v>
+        <v>1.0388787233184895</v>
       </c>
       <c r="N97" s="4">
-        <v>129.40720261608612</v>
+        <v>116.35441701167082</v>
       </c>
     </row>
     <row r="98">
@@ -12762,16 +12774,16 @@
         <v>134.0</v>
       </c>
       <c r="K98" s="4">
-        <v>133.31119012106313</v>
+        <v>141.23577148513135</v>
       </c>
       <c r="L98" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M98" s="6">
-        <v>0.9207391953901104</v>
+        <v>0.9463825493634996</v>
       </c>
       <c r="N98" s="4">
-        <v>123.37905218227479</v>
+        <v>126.81526161470894</v>
       </c>
     </row>
     <row r="99">
@@ -12820,16 +12832,16 @@
         <v>114.43</v>
       </c>
       <c r="K99" s="4">
-        <v>106.23382292548273</v>
+        <v>128.66089802326437</v>
       </c>
       <c r="L99" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M99" s="6">
-        <v>1.1554214519293404</v>
+        <v>1.0388787233184895</v>
       </c>
       <c r="N99" s="4">
-        <v>132.21487674427442</v>
+        <v>118.87889230933476</v>
       </c>
     </row>
     <row r="100">
@@ -12878,16 +12890,16 @@
         <v>134.0</v>
       </c>
       <c r="K100" s="4">
-        <v>133.31119012106313</v>
+        <v>141.23577148513135</v>
       </c>
       <c r="L100" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
       <c r="M100" s="6">
-        <v>0.9207391953901104</v>
+        <v>0.9463825493634996</v>
       </c>
       <c r="N100" s="4">
-        <v>123.37905218227479</v>
+        <v>126.81526161470894</v>
       </c>
     </row>
     <row r="101">
@@ -12936,16 +12948,16 @@
         <v>119.0</v>
       </c>
       <c r="K101" s="4">
-        <v>111.47285229808246</v>
+        <v>145.38258184831957</v>
       </c>
       <c r="L101" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M101" s="6">
-        <v>1.1023663442138323</v>
+        <v>0.9413096690765503</v>
       </c>
       <c r="N101" s="4">
-        <v>131.18159496144605</v>
+        <v>112.01585062010949</v>
       </c>
     </row>
     <row r="102">
@@ -12994,16 +13006,16 @@
         <v>107.25</v>
       </c>
       <c r="K102" s="4">
-        <v>105.90433306375704</v>
+        <v>132.3222914049477</v>
       </c>
       <c r="L102" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M102" s="6">
-        <v>1.1603294890016114</v>
+        <v>1.0342175045195687</v>
       </c>
       <c r="N102" s="4">
-        <v>124.44533769542282</v>
+        <v>110.91982735972374</v>
       </c>
     </row>
     <row r="103">
@@ -13052,16 +13064,16 @@
         <v>136.75</v>
       </c>
       <c r="K103" s="4">
-        <v>140.80796531259895</v>
+        <v>162.08574359104642</v>
       </c>
       <c r="L103" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M103" s="6">
-        <v>0.8727057478184473</v>
+        <v>0.8443063959679162</v>
       </c>
       <c r="N103" s="4">
-        <v>119.34251101417267</v>
+        <v>115.45889964861254</v>
       </c>
     </row>
     <row r="104">
@@ -13110,16 +13122,16 @@
         <v>123.25</v>
       </c>
       <c r="K104" s="4">
-        <v>133.39983923298843</v>
+        <v>147.5249422824168</v>
       </c>
       <c r="L104" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M104" s="6">
-        <v>0.9211699307395995</v>
+        <v>0.9276399495019295</v>
       </c>
       <c r="N104" s="4">
-        <v>113.53419396365564</v>
+        <v>114.3316237761128</v>
       </c>
     </row>
     <row r="105">
@@ -13168,16 +13180,16 @@
         <v>119.0</v>
       </c>
       <c r="K105" s="4">
-        <v>117.69733946950019</v>
+        <v>157.21513426867773</v>
       </c>
       <c r="L105" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M105" s="6">
-        <v>1.0440671065361635</v>
+        <v>0.8704634617126747</v>
       </c>
       <c r="N105" s="4">
-        <v>124.24398567780347</v>
+        <v>103.5851519438083</v>
       </c>
     </row>
     <row r="106">
@@ -13226,16 +13238,16 @@
         <v>107.25</v>
       </c>
       <c r="K106" s="4">
-        <v>111.81788195896411</v>
+        <v>143.09187899601477</v>
       </c>
       <c r="L106" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M106" s="6">
-        <v>1.0989648392018612</v>
+        <v>0.9563787335055374</v>
       </c>
       <c r="N106" s="4">
-        <v>117.86397900439961</v>
+        <v>102.57161916846889</v>
       </c>
     </row>
     <row r="107">
@@ -13284,16 +13296,16 @@
         <v>120.71</v>
       </c>
       <c r="K107" s="4">
-        <v>111.03122313124614</v>
+        <v>145.38258184831957</v>
       </c>
       <c r="L107" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M107" s="6">
-        <v>1.1067510309390076</v>
+        <v>0.9413096690765503</v>
       </c>
       <c r="N107" s="4">
-        <v>133.5959169446476</v>
+        <v>113.62549015423039</v>
       </c>
     </row>
     <row r="108">
@@ -13342,16 +13354,16 @@
         <v>108.71</v>
       </c>
       <c r="K108" s="4">
-        <v>105.90433306375704</v>
+        <v>132.3222914049477</v>
       </c>
       <c r="L108" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M108" s="6">
-        <v>1.1603294890016114</v>
+        <v>1.0342175045195687</v>
       </c>
       <c r="N108" s="4">
-        <v>126.13941874936516</v>
+        <v>112.4297849163223</v>
       </c>
     </row>
     <row r="109">
@@ -13400,16 +13412,16 @@
         <v>140.29</v>
       </c>
       <c r="K109" s="4">
-        <v>140.25011734223722</v>
+        <v>162.08574359104642</v>
       </c>
       <c r="L109" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M109" s="6">
-        <v>0.8761769543983005</v>
+        <v>0.8443063959679162</v>
       </c>
       <c r="N109" s="4">
-        <v>122.91886493253756</v>
+        <v>118.44774429033896</v>
       </c>
     </row>
     <row r="110">
@@ -13458,16 +13470,16 @@
         <v>126.43</v>
       </c>
       <c r="K110" s="4">
-        <v>133.39983923298843</v>
+        <v>147.5249422824168</v>
       </c>
       <c r="L110" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M110" s="6">
-        <v>0.9211699307395995</v>
+        <v>0.9276399495019295</v>
       </c>
       <c r="N110" s="4">
-        <v>116.46351434340757</v>
+        <v>117.28151881552895</v>
       </c>
     </row>
     <row r="111">
@@ -13516,16 +13528,16 @@
         <v>120.71</v>
       </c>
       <c r="K111" s="4">
-        <v>117.23105035159215</v>
+        <v>157.21513426867773</v>
       </c>
       <c r="L111" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M111" s="6">
-        <v>1.0482199067429643</v>
+        <v>0.8704634617126747</v>
       </c>
       <c r="N111" s="4">
-        <v>126.5306249429432</v>
+        <v>105.07364446333696</v>
       </c>
     </row>
     <row r="112">
@@ -13574,16 +13586,16 @@
         <v>108.71</v>
       </c>
       <c r="K112" s="4">
-        <v>111.81788195896411</v>
+        <v>143.09187899601477</v>
       </c>
       <c r="L112" s="4">
-        <v>122.88392066692566</v>
+        <v>136.8500300091362</v>
       </c>
       <c r="M112" s="6">
-        <v>1.0989648392018612</v>
+        <v>0.9563787335055374</v>
       </c>
       <c r="N112" s="4">
-        <v>119.46846766963432</v>
+        <v>103.96793211938696</v>
       </c>
     </row>
   </sheetData>
@@ -13659,7 +13671,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <v>59.97577158285408</v>
+        <v>35.79981320938094</v>
       </c>
     </row>
     <row r="8">
@@ -13669,7 +13681,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <v>0.8842284171459198</v>
+        <v>25.060186790619056</v>
       </c>
     </row>
     <row r="9">
@@ -13679,7 +13691,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <v>122.7448379285657</v>
+        <v>133.66306947941928</v>
       </c>
     </row>
     <row r="10">
@@ -13689,7 +13701,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <v>62.76906634571162</v>
+        <v>97.86325627003833</v>
       </c>
     </row>
     <row r="11">
@@ -13711,81 +13723,81 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>subscore_location</t>
+          <t>star_rating</t>
         </is>
       </c>
       <c r="B13" s="4">
-        <v>0.08929645949405834</v>
+        <v>0.23636669603545163</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>room_size_sqm</t>
+          <t>facility__sun_loungers_or_beach_chairs</t>
         </is>
       </c>
       <c r="B14" s="4">
-        <v>0.07269365381880571</v>
+        <v>-0.07794140951721594</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>subscore_comfort</t>
+          <t>room_size_sqm</t>
         </is>
       </c>
       <c r="B15" s="4">
-        <v>0.07055837185899178</v>
+        <v>0.07772012185133068</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>facility__free_toiletries</t>
+          <t>amenity__private_apartment_in_building</t>
         </is>
       </c>
       <c r="B16" s="4">
-        <v>0.054870486755297807</v>
+        <v>0.055805792600977386</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>facility__laundry_additional_charge</t>
+          <t>amenity__free_toiletries</t>
         </is>
       </c>
       <c r="B17" s="4">
-        <v>0.04794153024297472</v>
+        <v>0.03584584984733296</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>amenity__dining_area</t>
+          <t>facility__beachfront</t>
         </is>
       </c>
       <c r="B18" s="4">
-        <v>0.03874755113585365</v>
+        <v>0.027933792382918324</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>review_score</t>
+          <t>subscore_location</t>
         </is>
       </c>
       <c r="B19" s="4">
-        <v>0.03589691121488158</v>
+        <v>0.020546126585844718</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>review_count</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B20" s="4">
-        <v>-0.03270767532155847</v>
+        <v>-0.020280208138876044</v>
       </c>
     </row>
     <row r="21">
@@ -13795,17 +13807,17 @@
         </is>
       </c>
       <c r="B21" s="4">
-        <v>0.032535023956222875</v>
+        <v>-0.019134197254294598</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>facility__car_hire</t>
+          <t>review_count</t>
         </is>
       </c>
       <c r="B22" s="4">
-        <v>0.03209535247965844</v>
+        <v>-0.017830935829421003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>